<commit_message>
feat: implement solver core logic and generate comprehensive model evaluation results and visualizations
</commit_message>
<xml_diff>
--- a/results/eps_constraint/pareto_results_K20_risk.xlsx
+++ b/results/eps_constraint/pareto_results_K20_risk.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,11 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>avg_cov</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>selected_sites</t>
         </is>
       </c>
@@ -453,14 +458,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>31.0118</v>
+        <v>22.7685</v>
       </c>
       <c r="D2" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.8018</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.9561</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4,16,25,58,60,62,70,83</t>
         </is>
       </c>
     </row>
@@ -474,14 +482,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D3" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -495,14 +506,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D4" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -516,14 +530,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D5" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -537,14 +554,17 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D6" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -558,14 +578,17 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D7" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -579,14 +602,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D8" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -600,14 +626,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.0118</v>
+        <v>22.6771</v>
       </c>
       <c r="D9" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>0.9627</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.9137</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>3,4,16,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -621,14 +650,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D10" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -642,14 +674,17 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D11" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -663,14 +698,17 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D12" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -684,14 +722,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D13" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -705,14 +746,17 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D14" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -726,14 +770,17 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31.0118</v>
+        <v>22.4215</v>
       </c>
       <c r="D15" t="n">
-        <v>1.0893</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,100,117,127,135,140</t>
+        <v>1.0871</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.8886</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>3,4,11,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -747,14 +794,17 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30.9757</v>
+        <v>22.3781</v>
       </c>
       <c r="D16" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,103,117,127,135,140</t>
+        <v>1.1607</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.8863</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3,4,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -768,14 +818,17 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>30.9757</v>
+        <v>22.3781</v>
       </c>
       <c r="D17" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,103,117,127,135,140</t>
+        <v>1.1607</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.8863</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>3,4,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -789,14 +842,17 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30.9757</v>
+        <v>22.3781</v>
       </c>
       <c r="D18" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,103,117,127,135,140</t>
+        <v>1.1607</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.8863</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>3,4,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -810,14 +866,17 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30.9757</v>
+        <v>22.3781</v>
       </c>
       <c r="D19" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,103,117,127,135,140</t>
+        <v>1.1607</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.8863</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3,4,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -831,14 +890,17 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>30.935</v>
+        <v>22.2246</v>
       </c>
       <c r="D20" t="n">
-        <v>1.1936</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,42,54,55,59,60,61,62,63,70,83,103,117,127,135,140</t>
+        <v>1.2347</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2.8653</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>4,5,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>
@@ -852,14 +914,17 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30.8559</v>
+        <v>22.2246</v>
       </c>
       <c r="D21" t="n">
-        <v>1.2383</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>3,4,16,25,30,35,54,55,59,60,61,62,63,70,83,108,117,127,135,140</t>
+        <v>1.2347</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.8653</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>4,5,8,25,58,60,70,83</t>
         </is>
       </c>
     </row>

</xml_diff>